<commit_message>
Make sample import rows unique per person
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRRBvkKjt3A9PgQv7tKcVq
</commit_message>
<xml_diff>
--- a/project/sample-imports/doctors-sample.xlsx
+++ b/project/sample-imports/doctors-sample.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="86">
   <si>
     <t>staff_number</t>
   </si>
@@ -85,7 +85,7 @@
     <t>General Medicine</t>
   </si>
   <si>
-    <t>MBChB</t>
+    <t>MBChB;DipPEC</t>
   </si>
   <si>
     <t>English;isiZulu</t>
@@ -127,6 +127,24 @@
     <t>Cardiology</t>
   </si>
   <si>
+    <t>MBChB;MMed Internal Medicine;FCP(SA)</t>
+  </si>
+  <si>
+    <t>English;Sesotho;Afrikaans</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>07:00</t>
+  </si>
+  <si>
+    <t>15:00</t>
+  </si>
+  <si>
+    <t>Mon;Wed;Fri</t>
+  </si>
+  <si>
     <t>DR-2003</t>
   </si>
   <si>
@@ -151,6 +169,24 @@
     <t>Paediatrics</t>
   </si>
   <si>
+    <t>MBChB;DCH(SA);MMed Paediatrics</t>
+  </si>
+  <si>
+    <t>English;Afrikaans</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>09:00</t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>Tue;Wed;Thu;Sat</t>
+  </si>
+  <si>
     <t>DR-2004</t>
   </si>
   <si>
@@ -175,6 +211,24 @@
     <t>Dermatology</t>
   </si>
   <si>
+    <t>MBChB;FC Derm(SA)</t>
+  </si>
+  <si>
+    <t>English;isiXhosa;Setswana</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>10:00</t>
+  </si>
+  <si>
+    <t>18:00</t>
+  </si>
+  <si>
+    <t>Mon;Tue;Thu;Fri</t>
+  </si>
+  <si>
     <t>DR-2005</t>
   </si>
   <si>
@@ -200,6 +254,21 @@
   </si>
   <si>
     <t>Emergency</t>
+  </si>
+  <si>
+    <t>BCur;Diploma Emergency Nursing</t>
+  </si>
+  <si>
+    <t>English;isiZulu;Siswati</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>23:00</t>
+  </si>
+  <si>
+    <t>Fri;Sat;Sun</t>
   </si>
 </sst>
 </file>
@@ -702,163 +771,163 @@
         <v>37</v>
       </c>
       <c r="J3" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="K3" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="L3" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="M3" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="N3" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="O3" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D4" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H4" t="s">
         <v>22</v>
       </c>
       <c r="I4" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="J4" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="K4" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="L4" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="M4" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="N4" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="O4" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="G5" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="H5" t="s">
         <v>22</v>
       </c>
       <c r="I5" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="J5" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="K5" t="s">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="L5" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
       <c r="M5" t="s">
-        <v>27</v>
+        <v>69</v>
       </c>
       <c r="N5" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="O5" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="E6" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="F6" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="G6" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="H6" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="I6" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="J6" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="K6" t="s">
-        <v>25</v>
+        <v>82</v>
       </c>
       <c r="L6" t="s">
-        <v>26</v>
+        <v>83</v>
       </c>
       <c r="M6" t="s">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="N6" t="s">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="O6" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add UAT import spreadsheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRRBvkKjt3A9PgQv7tKcVq
</commit_message>
<xml_diff>
--- a/project/sample-imports/doctors-sample.xlsx
+++ b/project/sample-imports/doctors-sample.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="63">
   <si>
     <t>staff_number</t>
   </si>
@@ -58,7 +58,7 @@
     <t>shift_days</t>
   </si>
   <si>
-    <t>DR-2001</t>
+    <t>UAT-D-01</t>
   </si>
   <si>
     <t>Mayo</t>
@@ -67,13 +67,13 @@
     <t>Maziya</t>
   </si>
   <si>
-    <t>maziyamayo7@gmail.com</t>
-  </si>
-  <si>
-    <t>0711110001</t>
-  </si>
-  <si>
-    <t>MP0200001</t>
+    <t>maziyamayo7+doctor1@gmail.com</t>
+  </si>
+  <si>
+    <t>0715550001</t>
+  </si>
+  <si>
+    <t>MP0555001</t>
   </si>
   <si>
     <t>General Practitioner</t>
@@ -85,7 +85,7 @@
     <t>General Medicine</t>
   </si>
   <si>
-    <t>MBChB;DipPEC</t>
+    <t>MBChB</t>
   </si>
   <si>
     <t>English;isiZulu</t>
@@ -103,7 +103,7 @@
     <t>Mon;Tue;Wed;Thu;Fri</t>
   </si>
   <si>
-    <t>DR-2002</t>
+    <t>UAT-D-02</t>
   </si>
   <si>
     <t>Anele</t>
@@ -112,13 +112,13 @@
     <t>Zulu</t>
   </si>
   <si>
-    <t>anele.zulu.test@example.com</t>
-  </si>
-  <si>
-    <t>0711110002</t>
-  </si>
-  <si>
-    <t>MP0200002</t>
+    <t>makabmahlalela+doctor2@gmail.com</t>
+  </si>
+  <si>
+    <t>0715550002</t>
+  </si>
+  <si>
+    <t>MP0555002</t>
   </si>
   <si>
     <t>Cardiologist</t>
@@ -127,25 +127,7 @@
     <t>Cardiology</t>
   </si>
   <si>
-    <t>MBChB;MMed Internal Medicine;FCP(SA)</t>
-  </si>
-  <si>
-    <t>English;Sesotho;Afrikaans</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>07:00</t>
-  </si>
-  <si>
-    <t>15:00</t>
-  </si>
-  <si>
-    <t>Mon;Wed;Fri</t>
-  </si>
-  <si>
-    <t>DR-2003</t>
+    <t>UAT-D-03</t>
   </si>
   <si>
     <t>Ruth</t>
@@ -154,13 +136,13 @@
     <t>Smit</t>
   </si>
   <si>
-    <t>ruth.smit.test@example.com</t>
-  </si>
-  <si>
-    <t>0711110003</t>
-  </si>
-  <si>
-    <t>MP0200003</t>
+    <t>maziyamayo7+doctor3@gmail.com</t>
+  </si>
+  <si>
+    <t>0715550003</t>
+  </si>
+  <si>
+    <t>MP0555003</t>
   </si>
   <si>
     <t>Paediatrician</t>
@@ -169,25 +151,7 @@
     <t>Paediatrics</t>
   </si>
   <si>
-    <t>MBChB;DCH(SA);MMed Paediatrics</t>
-  </si>
-  <si>
-    <t>English;Afrikaans</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>09:00</t>
-  </si>
-  <si>
-    <t>17:00</t>
-  </si>
-  <si>
-    <t>Tue;Wed;Thu;Sat</t>
-  </si>
-  <si>
-    <t>DR-2004</t>
+    <t>UAT-D-04</t>
   </si>
   <si>
     <t>Kabelo</t>
@@ -196,13 +160,13 @@
     <t>Mokoena</t>
   </si>
   <si>
-    <t>kabelo.mokoena.test@example.com</t>
-  </si>
-  <si>
-    <t>0711110004</t>
-  </si>
-  <si>
-    <t>MP0200004</t>
+    <t>makabmahlalela+doctor4@gmail.com</t>
+  </si>
+  <si>
+    <t>0715550004</t>
+  </si>
+  <si>
+    <t>MP0555004</t>
   </si>
   <si>
     <t>Dermatologist</t>
@@ -211,25 +175,7 @@
     <t>Dermatology</t>
   </si>
   <si>
-    <t>MBChB;FC Derm(SA)</t>
-  </si>
-  <si>
-    <t>English;isiXhosa;Setswana</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>10:00</t>
-  </si>
-  <si>
-    <t>18:00</t>
-  </si>
-  <si>
-    <t>Mon;Tue;Thu;Fri</t>
-  </si>
-  <si>
-    <t>DR-2005</t>
+    <t>UAT-D-05</t>
   </si>
   <si>
     <t>Zanele</t>
@@ -238,13 +184,13 @@
     <t>Ndlovu</t>
   </si>
   <si>
-    <t>zanele.ndlovu.test@example.com</t>
-  </si>
-  <si>
-    <t>0711110005</t>
-  </si>
-  <si>
-    <t>MP0200005</t>
+    <t>maziyamayo7+doctor5@gmail.com</t>
+  </si>
+  <si>
+    <t>0715550005</t>
+  </si>
+  <si>
+    <t>MP0555005</t>
   </si>
   <si>
     <t>Nurse Practitioner</t>
@@ -254,21 +200,6 @@
   </si>
   <si>
     <t>Emergency</t>
-  </si>
-  <si>
-    <t>BCur;Diploma Emergency Nursing</t>
-  </si>
-  <si>
-    <t>English;isiZulu;Siswati</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>23:00</t>
-  </si>
-  <si>
-    <t>Fri;Sat;Sun</t>
   </si>
 </sst>
 </file>
@@ -771,163 +702,163 @@
         <v>37</v>
       </c>
       <c r="J3" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="K3" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="L3" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="M3" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="N3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="O3" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" t="s">
         <v>44</v>
-      </c>
-      <c r="B4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4" t="s">
-        <v>48</v>
-      </c>
-      <c r="F4" t="s">
-        <v>49</v>
-      </c>
-      <c r="G4" t="s">
-        <v>50</v>
       </c>
       <c r="H4" t="s">
         <v>22</v>
       </c>
       <c r="I4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="J4" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="K4" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="L4" t="s">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="M4" t="s">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="N4" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="O4" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="G5" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="H5" t="s">
         <v>22</v>
       </c>
       <c r="I5" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="J5" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="K5" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="L5" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="M5" t="s">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="N5" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="O5" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="C6" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="E6" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="G6" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="I6" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="J6" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="K6" t="s">
-        <v>82</v>
+        <v>25</v>
       </c>
       <c r="L6" t="s">
-        <v>83</v>
+        <v>26</v>
       </c>
       <c r="M6" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="N6" t="s">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="O6" t="s">
-        <v>85</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>